<commit_message>
docs(tabs): config guides for narrative, What if, delivery modes and module tabs; island paths resolve against the config
</commit_message>
<xml_diff>
--- a/modules/catdriver/docs/templates/CatDriver_Config_Template.xlsx
+++ b/modules/catdriver/docs/templates/CatDriver_Config_Template.xlsx
@@ -110,30 +110,24 @@
     <t xml:space="preserve">multinomial_mode</t>
   </si>
   <si>
-    <t xml:space="preserve">Required if outcome_type=multinomial. Determines how multinomial outcomes are modelled.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">baseline_category, all_pairwise, one_vs_all, or per_outcome</t>
-  </si>
-  <si>
-    <t xml:space="preserve">target_outcome_level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Required if multinomial_mode=one_vs_all. The specific outcome level to compare against all others.</t>
+    <t xml:space="preserve">baseline_category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required if outcome_type=multinomial. One mode is implemented: every outcome level is compared with one reference level.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REFERENCE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reference_category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference/baseline category for comparisons. If blank, the first category in the declared Order is used (alphabetically first when no Order is given), NOT the most frequent.</t>
   </si>
   <si>
     <t xml:space="preserve">A value that appears in the outcome variable</t>
   </si>
   <si>
-    <t xml:space="preserve">REFERENCE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reference_category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference/baseline category for comparisons. If blank, the most frequent category is used.</t>
-  </si>
-  <si>
     <t xml:space="preserve">allow_missing_reference</t>
   </si>
   <si>
@@ -248,7 +242,7 @@
     <t xml:space="preserve">Generate_Stats_Pack</t>
   </si>
   <si>
-    <t xml:space="preserve">N</t>
+    <t xml:space="preserve">Y</t>
   </si>
   <si>
     <t xml:space="preserve">Generate a diagnostic stats pack workbook alongside main output. The stats pack provides a full audit trail of data received, methods used, assumptions, and reproducibility — designed for advanced partners and research statisticians. Output file is named {output}_stats_pack.xlsx.</t>
@@ -257,6 +251,12 @@
     <t xml:space="preserve">Y or N</t>
   </si>
   <si>
+    <t xml:space="preserve">v2_island</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Also write {output}_cd_island.json beside the Excel output, so a tabs report for the same project can carry a Categorical drivers tab. Point the tabs config's catdriver_island setting at that file. Off by default: a project with no tabs report has no use for it.</t>
+  </si>
+  <si>
     <t xml:space="preserve">probability_lifts</t>
   </si>
   <si>
@@ -410,7 +410,7 @@
     <t xml:space="preserve">[REQUIRED] Human-readable label for reports and output tables.</t>
   </si>
   <si>
-    <t xml:space="preserve">[Optional] Semicolon-separated category order for ordinal variables (LOW to HIGH). Leave blank for nominal.</t>
+    <t xml:space="preserve">[Optional] Semicolon-separated category order for ordinal variables (LOW to HIGH). REQUIRED for an ordinal outcome: without it the categories are sorted alphabetically and the model fits the wrong order. Leave blank for nominal.</t>
   </si>
   <si>
     <t xml:space="preserve">satisfaction</t>
@@ -488,7 +488,7 @@
     <t xml:space="preserve">[REQUIRED] Driver variable name. Must match a VariableName with Type=Driver in the Variables sheet.</t>
   </si>
   <si>
-    <t xml:space="preserve">[REQUIRED] Statistical type: ordinal (ordered categories), nominal (unordered categories), categorical (generic), control_only (included as covariate, not reported as driver).</t>
+    <t xml:space="preserve">[REQUIRED] Statistical type: categorical (unordered categories), ordinal (ordered categories, needs levels_order), binary (two categories), control_only (included as a covariate, not reported as a driver).</t>
   </si>
   <si>
     <t xml:space="preserve">[Optional] Semicolon-separated level order LOW to HIGH for ordinal drivers. Required when type=ordinal.</t>
@@ -562,7 +562,7 @@
   <si>
     <t xml:space="preserve">The analysis uses categorical key driver modelling with:
 - Ordinal logistic regression
-- SHAP-based importance decomposition
+- Type II Wald chi-square importance ranking
 - Bootstrap confidence intervals (n=500)</t>
   </si>
   <si>
@@ -1230,213 +1230,213 @@
         <v>30</v>
       </c>
       <c r="B13" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" s="14" t="s">
+      <c r="C15" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" s="13" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="s">
+      <c r="E15" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="s">
         <v>37</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D17" s="13" t="s">
+      <c r="A17" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="E17" s="14" t="s">
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="s">
+      <c r="B18" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
+      <c r="C18" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>45</v>
+        <v>46</v>
+      </c>
+      <c r="B19" s="11" t="n">
+        <v>10</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B20" s="11" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C20" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="B21" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="C21" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D21" s="13" t="s">
+      <c r="A21" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="E21" s="14" t="s">
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="s">
+      <c r="B22" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
+      <c r="E22" s="14" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B23" s="11" t="n">
-        <v>30</v>
+        <v>0.95</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B24" s="11" t="n">
-        <v>0.95</v>
+        <v>50</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="B25" s="11" t="n">
-        <v>50</v>
-      </c>
-      <c r="C25" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D25" s="13" t="s">
+      <c r="A25" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="E25" s="14" t="s">
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="s">
+      <c r="B26" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
+      <c r="C26" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>4</v>
@@ -1445,15 +1445,15 @@
         <v>67</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="B28" s="11" t="s">
-        <v>40</v>
+      <c r="B28" s="11" t="n">
+        <v>200</v>
       </c>
       <c r="C28" s="16" t="s">
         <v>4</v>
@@ -1462,67 +1462,67 @@
         <v>69</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>42</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="B29" s="11" t="n">
-        <v>200</v>
-      </c>
-      <c r="C29" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D29" s="13" t="s">
+      <c r="A29" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="E29" s="14" t="s">
+      <c r="B29" s="9"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="s">
+      <c r="B30" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D30" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="B30" s="9"/>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
+      <c r="E30" s="14" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="15" t="s">
         <v>74</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="C31" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>42</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="15" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>77</v>
+        <v>38</v>
       </c>
       <c r="C32" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>79</v>
+        <v>40</v>
       </c>
     </row>
     <row r="33">
@@ -1530,7 +1530,7 @@
         <v>80</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C33" s="16" t="s">
         <v>4</v>
@@ -1539,7 +1539,7 @@
         <v>81</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34">
@@ -1735,7 +1735,7 @@
         <v>112</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="46">
@@ -1743,7 +1743,7 @@
         <v>113</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C46" s="16" t="s">
         <v>4</v>
@@ -1752,7 +1752,7 @@
         <v>114</v>
       </c>
       <c r="E46" s="14" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="47">
@@ -1822,36 +1822,36 @@
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A29:E29"/>
     <mergeCell ref="A43:E43"/>
     <mergeCell ref="A47:E47"/>
   </mergeCells>
   <dataValidations count="7">
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B20:B20">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B19:B19">
       <formula1>1</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B21:B21">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B20:B20">
       <formula1>1</formula1>
       <formula2>50</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B23:B23">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B22:B22">
       <formula1>10</formula1>
       <formula2>10000</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B24:B24">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B23:B23">
       <formula1>0.8</formula1>
       <formula2>0.99</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B25:B25">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B24:B24">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B29:B29">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B28:B28">
       <formula1>50</formula1>
       <formula2>10000</formula2>
     </dataValidation>
@@ -1864,7 +1864,7 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="10">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="11">
         <x14:dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"binary,ordinal,multinomial"</xm:f>
@@ -1873,7 +1873,7 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>"baseline_category,all_pairwise,one_vs_all,per_outcome"</xm:f>
+            <xm:f>"baseline_category"</xm:f>
           </x14:formula1>
           <xm:sqref>B13:B13</xm:sqref>
         </x14:dataValidation>
@@ -1881,13 +1881,19 @@
           <x14:formula1>
             <xm:f>"TRUE,FALSE"</xm:f>
           </x14:formula1>
-          <xm:sqref>B17:B17</xm:sqref>
+          <xm:sqref>B16:B16</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"warn_only,collapse_to_other,drop_level,error"</xm:f>
           </x14:formula1>
-          <xm:sqref>B19:B19</xm:sqref>
+          <xm:sqref>B18:B18</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>B26:B26</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
@@ -1899,17 +1905,17 @@
           <x14:formula1>
             <xm:f>"TRUE,FALSE"</xm:f>
           </x14:formula1>
-          <xm:sqref>B28:B28</xm:sqref>
+          <xm:sqref>B30:B30</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>"TRUE,FALSE"</xm:f>
+            <xm:f>"Y,N"</xm:f>
           </x14:formula1>
           <xm:sqref>B31:B31</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>"Y,N"</xm:f>
+            <xm:f>"TRUE,FALSE"</xm:f>
           </x14:formula1>
           <xm:sqref>B32:B32</xm:sqref>
         </x14:dataValidation>
@@ -2292,7 +2298,7 @@
         <v>155</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
@@ -2547,7 +2553,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>"ordinal,nominal,categorical,control_only"</xm:f>
+            <xm:f>"categorical,ordinal,binary,control_only"</xm:f>
           </x14:formula1>
           <xm:sqref>B5:B27</xm:sqref>
         </x14:dataValidation>

</xml_diff>